<commit_message>
skill v1p3(format not good) and rtm
</commit_message>
<xml_diff>
--- a/RTM_TBUS_Generated.xlsx
+++ b/RTM_TBUS_Generated.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="23">
+  <fonts count="25">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -192,6 +192,14 @@
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="35">
@@ -815,7 +823,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -935,6 +943,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2841,36 +2867,36 @@
       </c>
     </row>
     <row r="3" ht="61" customHeight="1" s="31">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="45" t="inlineStr">
         <is>
           <t>CHK_001</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="45" t="inlineStr">
         <is>
           <t>clk_freq_check</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="46" t="inlineStr">
         <is>
           <t>1.检查频率值是否正确：连续采集clk_i时钟上升沿和下降沿并计算实际频率/周期，判断是否处于目标频率的允许误差范围内（100MHz ±1%）；
 2.检查时钟稳定性：通过连续采样周期，对比相邻两个周期的频率偏差是否在3%内。</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n"/>
+      <c r="D3" s="45" t="n"/>
     </row>
     <row r="4" ht="155" customHeight="1" s="31">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="45" t="inlineStr">
         <is>
           <t>CHK_002</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="45" t="inlineStr">
         <is>
           <t>reset_check</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="46" t="inlineStr">
         <is>
           <t>在rst_ni释放后的每个cycle，检查模块复位状态：
 1.状态机处于IDLE状态；
@@ -2881,20 +2907,20 @@
 6.协议上下文和错误状态已清空。</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n"/>
+      <c r="D4" s="45" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="45" t="inlineStr">
         <is>
           <t>CHK_003</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="45" t="inlineStr">
         <is>
           <t>csr_access_check</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="46" t="inlineStr">
         <is>
           <t>检查CSR寄存器访问正确性：
 1.VERSION寄存器(0x00)：只读，返回版本号值；
@@ -2904,20 +2930,20 @@
 5.非法CSR地址返回STS_BAD_REG(0x02)。</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n"/>
+      <c r="D5" s="45" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="45" t="inlineStr">
         <is>
           <t>CHK_004</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="45" t="inlineStr">
         <is>
           <t>test_mode_check</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="46" t="inlineStr">
         <is>
           <t>检查测试模式工作条件：
 1.test_mode_i=1且CTRL.EN=1时，模块允许执行功能命令；
@@ -2926,20 +2952,20 @@
 4.半双工请求/响应模式正常工作，pcs_n_i定义帧边界。</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n"/>
+      <c r="D6" s="45" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="45" t="inlineStr">
         <is>
           <t>CHK_005</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="45" t="inlineStr">
         <is>
           <t>lane_mode_check</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="46" t="inlineStr">
         <is>
           <t>检查lane模式切换正确性：
 1.LANE_MODE=00时，使用pdi_i[0]/pdo_o[0]进行1-bit传输；
@@ -2949,20 +2975,20 @@
 5.不支持8-bit/16-bit模式（MVP限制）。</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n"/>
+      <c r="D7" s="45" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="45" t="inlineStr">
         <is>
           <t>CHK_006</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="45" t="inlineStr">
         <is>
           <t>data_interface_check</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="46" t="inlineStr">
         <is>
           <t>检查数据接口传输正确性：
 1.pcs_n_i=1表示空闲，拉低后开始接收请求；
@@ -2972,20 +2998,20 @@
 5.数据按MSB first顺序传输。</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n"/>
+      <c r="D8" s="45" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="45" t="inlineStr">
         <is>
           <t>CHK_007</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="45" t="inlineStr">
         <is>
           <t>protocol_timing_check</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="46" t="inlineStr">
         <is>
           <t>检查协议时序正确性：
 1.请求阶段：ATE驱动pdi_i输入数据；
@@ -2996,20 +3022,20 @@
 6.pcs_n_i在请求未收满时提前拉高产生帧错误STS_FRAME_ERR(0x06)。</t>
         </is>
       </c>
-      <c r="D9" s="4" t="n"/>
+      <c r="D9" s="45" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="45" t="inlineStr">
         <is>
           <t>CHK_008</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="45" t="inlineStr">
         <is>
           <t>opcode_decode_check</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="46" t="inlineStr">
         <is>
           <t>检查opcode译码正确性：
 1.opcode=0x10 WR_CSR：CSR写命令，帧格式为opcode+addr+wdata；
@@ -3020,20 +3046,20 @@
 6.前端收满8bit opcode后确定期望帧长。</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n"/>
+      <c r="D10" s="45" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="45" t="inlineStr">
         <is>
           <t>CHK_009</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="45" t="inlineStr">
         <is>
           <t>ctrl_config_check</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="46" t="inlineStr">
         <is>
           <t>检查CTRL寄存器配置生效：
 1.CTRL.EN=1：模块使能，允许执行命令；
@@ -3044,20 +3070,20 @@
 6.CTRL.SOFT_RST写1：触发软复位，清零协议上下文，恢复LANE_MODE=00默认值。</t>
         </is>
       </c>
-      <c r="D11" s="4" t="n"/>
+      <c r="D11" s="45" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="45" t="inlineStr">
         <is>
           <t>CHK_010</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="45" t="inlineStr">
         <is>
           <t>status_polling_check</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="46" t="inlineStr">
         <is>
           <t>检查状态查询机制：
 1.STATUS[0] BUSY：当前有事务执行时置1；
@@ -3071,20 +3097,20 @@
 9.MVP版本无独立中断输出，通过轮询STATUS/LAST_ERR获取状态。</t>
         </is>
       </c>
-      <c r="D12" s="4" t="n"/>
+      <c r="D12" s="45" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="45" t="inlineStr">
         <is>
           <t>CHK_011</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="45" t="inlineStr">
         <is>
           <t>error_handling_check</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="46" t="inlineStr">
         <is>
           <t>检查异常检测与处理：
 1.STS_BAD_OPCODE(0x01)：opcode非0x10/0x11/0x20/0x21；
@@ -3099,19 +3125,20 @@
 10.LAST_ERR更新为最近错误码。</t>
         </is>
       </c>
+      <c r="D13" s="45" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="45" t="inlineStr">
         <is>
           <t>CHK_012</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="45" t="inlineStr">
         <is>
           <t>low_power_check</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="46" t="inlineStr">
         <is>
           <t>检查低功耗设计行为：
 1.pcs_n_i=1空闲态时，接收移位寄存器不更新；
@@ -3121,19 +3148,20 @@
 5.仅在RX/TX/WAIT_AHB相关状态翻转关键寄存器。</t>
         </is>
       </c>
+      <c r="D14" s="45" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="45" t="inlineStr">
         <is>
           <t>CHK_013</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="45" t="inlineStr">
         <is>
           <t>performance_check</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="46" t="inlineStr">
         <is>
           <t>检查性能指标：
 1.目标频率：clk_i=100MHz稳定工作；
@@ -3144,19 +3172,20 @@
 6.AHB接口：32bit字访问，地址4Byte对齐。</t>
         </is>
       </c>
+      <c r="D15" s="45" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="47" t="inlineStr">
         <is>
           <t>CHK_014</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="45" t="inlineStr">
         <is>
           <t>dfx_observable_check</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="46" t="inlineStr">
         <is>
           <t>检查调试可观测点：
 1.状态机状态可观测；
@@ -3170,19 +3199,20 @@
 9.关键接口信号可采集：pcs_n_i, pdi_i, pdo_o, pdo_oe_o。</t>
         </is>
       </c>
+      <c r="D16" s="45" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1" s="31">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="45" t="inlineStr">
         <is>
           <t>CHK_015</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="45" t="inlineStr">
         <is>
           <t>memory_map_check</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="46" t="inlineStr">
         <is>
           <t>检查存储映射：
 1.模块CSR通过协议命令访问，不进入SoC AHB memory map；
@@ -3192,19 +3222,20 @@
 5.AHB目标地址范围由SoC顶层约束。</t>
         </is>
       </c>
+      <c r="D17" s="45" t="n"/>
     </row>
     <row r="18" ht="70" customHeight="1" s="31">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="45" t="inlineStr">
         <is>
           <t>CHK_016</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="45" t="inlineStr">
         <is>
           <t>ahb_interface_check</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="46" t="inlineStr">
         <is>
           <t>检查AHB-Lite Master接口合规性：
 1.haddr_o：32bit地址输出；
@@ -3220,9 +3251,10 @@
 11.不支持outstanding，当前事务完成前不得发起新请求。</t>
         </is>
       </c>
+      <c r="D18" s="45" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="48" t="inlineStr">
         <is>
           <t>填写要求</t>
         </is>
@@ -3250,8 +3282,9 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>1、需要定性+定量描述，需具体到check的信号、取值 
-2、和DV SPEC中Checker方案描述的区别 — RTM中描述check的内容，DV SPEC中描述checker的实现方案(例如是通过SVA实现还是scoreboard实时数据比对，还是文件对比)</t>
+          <t xml:space="preserve">1、需要定性+定量描述，需具体到check的信号、取值 
+2、和DV SPEC中Checker方案描述的区别 — RTM中描述check的内容，DV SPEC中描述checker的实现方案(例如是通过SVA实现还是scoreboard实时数据比对，还是文件对比)
+</t>
         </is>
       </c>
       <c r="C21" s="29" t="n"/>
@@ -3260,10 +3293,14 @@
     <row r="22">
       <c r="A22" s="6" t="n"/>
       <c r="B22" s="6" t="n"/>
+      <c r="C22" s="29" t="n"/>
+      <c r="D22" s="30" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="6" t="n"/>
+      <c r="C23" s="29" t="n"/>
+      <c r="D23" s="30" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3324,17 +3361,17 @@
       </c>
     </row>
     <row r="3" ht="98" customHeight="1" s="31">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="49" t="inlineStr">
         <is>
           <t>DV_TC_001</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="49" t="inlineStr">
         <is>
           <t>tbus_clk_freq_test</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.配置clk_i时钟频率为100MHz；
@@ -3354,20 +3391,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n"/>
+      <c r="D3" s="49" t="n"/>
     </row>
     <row r="4" ht="192" customHeight="1" s="31">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="49" t="inlineStr">
         <is>
           <t>DV_TC_002</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="49" t="inlineStr">
         <is>
           <t>tbus_reset_test</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.初始状态rst_ni为低，模块处于复位状态；
@@ -3389,20 +3426,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n"/>
+      <c r="D4" s="49" t="n"/>
     </row>
     <row r="5" ht="55" customHeight="1" s="31">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="49" t="inlineStr">
         <is>
           <t>DV_TC_003</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="49" t="inlineStr">
         <is>
           <t>tbus_csr_access_test</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.test_mode_i=1，CTRL.EN=1；
@@ -3424,20 +3461,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n"/>
+      <c r="D5" s="49" t="n"/>
     </row>
     <row r="6" ht="26" customHeight="1" s="31">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="49" t="inlineStr">
         <is>
           <t>DV_TC_004</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="49" t="inlineStr">
         <is>
           <t>tbus_test_mode_test</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.test_mode_i=1；
@@ -3459,20 +3496,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n"/>
+      <c r="D6" s="49" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="49" t="inlineStr">
         <is>
           <t>DV_TC_005</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="49" t="inlineStr">
         <is>
           <t>tbus_lane_mode_test</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.test_mode_i=1，CTRL.EN=1；
@@ -3493,20 +3530,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n"/>
+      <c r="D7" s="49" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="49" t="inlineStr">
         <is>
           <t>DV_TC_006</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="49" t="inlineStr">
         <is>
           <t>tbus_data_interface_test</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.test_mode_i=1，CTRL.EN=1；
@@ -3527,20 +3564,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n"/>
+      <c r="D8" s="49" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="49" t="inlineStr">
         <is>
           <t>DV_TC_007</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="49" t="inlineStr">
         <is>
           <t>tbus_protocol_timing_test</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.test_mode_i=1，CTRL.EN=1；
@@ -3562,20 +3599,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
-      <c r="D9" s="4" t="n"/>
+      <c r="D9" s="49" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="49" t="inlineStr">
         <is>
           <t>DV_TC_008</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="49" t="inlineStr">
         <is>
           <t>tbus_opcode_test</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.test_mode_i=1，CTRL.EN=1；
@@ -3597,20 +3634,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n"/>
+      <c r="D10" s="49" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="49" t="inlineStr">
         <is>
           <t>DV_TC_009</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="49" t="inlineStr">
         <is>
           <t>tbus_ctrl_config_test</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.test_mode_i=1；
@@ -3631,20 +3668,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
-      <c r="D11" s="4" t="n"/>
+      <c r="D11" s="49" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="49" t="inlineStr">
         <is>
           <t>DV_TC_010</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="49" t="inlineStr">
         <is>
           <t>tbus_status_polling_test</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.test_mode_i=1，CTRL.EN=1；
@@ -3666,20 +3703,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
-      <c r="D12" s="4" t="n"/>
+      <c r="D12" s="49" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="49" t="inlineStr">
         <is>
           <t>DV_TC_011</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="49" t="inlineStr">
         <is>
           <t>tbus_error_handling_test</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.test_mode_i=1，CTRL.EN=1；
@@ -3702,19 +3739,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
+      <c r="D13" s="49" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="49" t="inlineStr">
         <is>
           <t>DV_TC_012</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="49" t="inlineStr">
         <is>
           <t>tbus_low_power_test</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.模块处于空闲态(test_mode_i=0或无有效任务)；
@@ -3735,19 +3773,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
+      <c r="D14" s="49" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="49" t="inlineStr">
         <is>
           <t>DV_TC_013</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="49" t="inlineStr">
         <is>
           <t>tbus_performance_test</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.配置clk_i=100MHz；
@@ -3770,19 +3809,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
+      <c r="D15" s="49" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="49" t="inlineStr">
         <is>
           <t>DV_TC_014</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="49" t="inlineStr">
         <is>
           <t>tbus_dfx_test</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.仿真环境；
@@ -3803,19 +3843,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
+      <c r="D16" s="49" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="49" t="inlineStr">
         <is>
           <t>DV_TC_015</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="49" t="inlineStr">
         <is>
           <t>tbus_memory_map_test</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.test_mode_i=1，CTRL.EN=1。
@@ -3837,19 +3878,20 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
+      <c r="D17" s="49" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="49" t="inlineStr">
         <is>
           <t>DV_TC_016</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="49" t="inlineStr">
         <is>
           <t>tbus_ahb_interface_test</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="50" t="inlineStr">
         <is>
           <t>配置条件：
 1.test_mode_i=1，CTRL.EN=1；
@@ -3882,6 +3924,7 @@
 直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
+      <c r="D18" s="49" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>